<commit_message>
5417 - Static file upload: --reupload and update bulk download files
</commit_message>
<xml_diff>
--- a/src/tools/uploadStaticFiles/staticFiles/fra/2025/dataDownload/6 Permanent forest estate en.xlsx
+++ b/src/tools/uploadStaticFiles/staticFiles/fra/2025/dataDownload/6 Permanent forest estate en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfao-my.sharepoint.com/personal/pengcheng_lai_fao_org/Documents/Desktop/worksheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfao-my.sharepoint.com/personal/pengcheng_lai_fao_org/Documents/Desktop/Update/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{9EB7299C-8445-45FA-928C-21125EB2985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B78550D-900F-47F3-94D3-702C715DA43D}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{9EB7299C-8445-45FA-928C-21125EB2985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06A64972-452A-46DE-ABA1-0DD5BCE4B625}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1670,9 +1670,6 @@
     <t>PCN</t>
   </si>
   <si>
-    <t>Pitcairn Islands</t>
-  </si>
-  <si>
     <t>WSM</t>
   </si>
   <si>
@@ -1879,6 +1876,9 @@
   </si>
   <si>
     <t>These analysis tables include data reported by countries and it is important to note that some of the regional totals may differ from the results presented in the FRA 2025 main report. The reason for this discrepancy is that in some cases, gap-filling was performed for missing values in order to obtain complete time series for the main report. Therefore, it is not always possible to reproduce the global, regional and subregional aggregates presented in the FRA 2025 main report by using the analysis tables.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pitcairn </t>
   </si>
 </sst>
 </file>
@@ -2396,6 +2396,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2412,25 +2430,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3088,7 +3088,7 @@
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1">
       <c r="A2" s="64" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B2" s="64"/>
       <c r="C2" s="64"/>
@@ -3149,7 +3149,7 @@
     </row>
     <row r="5" spans="1:17" ht="32.25" customHeight="1">
       <c r="A5" s="64" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -3191,7 +3191,7 @@
     </row>
     <row r="7" spans="1:17" ht="48" customHeight="1">
       <c r="A7" s="61" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B7" s="61"/>
       <c r="C7" s="61"/>
@@ -3254,7 +3254,7 @@
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="63" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B10" s="63"/>
       <c r="C10" s="63"/>
@@ -3363,17 +3363,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="A8:Q8"/>
-    <mergeCell ref="A9:Q9"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A83:Q83"/>
     <mergeCell ref="A89:Q89"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q3"/>
     <mergeCell ref="A4:Q4"/>
     <mergeCell ref="A5:Q5"/>
     <mergeCell ref="A6:Q6"/>
+    <mergeCell ref="A7:Q7"/>
+    <mergeCell ref="A8:Q8"/>
+    <mergeCell ref="A9:Q9"/>
+    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A83:Q83"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3439,62 +3439,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" s="7" customFormat="1" ht="24" customHeight="1">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74" t="s">
-        <v>529</v>
-      </c>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="74"/>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
-      <c r="S1" s="74"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="74"/>
-      <c r="V1" s="74"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="74"/>
-      <c r="AF1" s="74"/>
-      <c r="AG1" s="74"/>
-      <c r="AH1" s="74"/>
-      <c r="AI1" s="74"/>
-      <c r="AJ1" s="74"/>
-      <c r="AK1" s="74"/>
-      <c r="AL1" s="74"/>
-      <c r="AM1" s="74"/>
-      <c r="AN1" s="74"/>
-      <c r="AO1" s="74"/>
-      <c r="AP1" s="74"/>
-      <c r="AQ1" s="74"/>
-      <c r="AR1" s="74"/>
-      <c r="AS1" s="74"/>
-      <c r="AT1" s="74"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67" t="s">
+        <v>528</v>
+      </c>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
     </row>
     <row r="2" spans="1:46">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="71" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="72" t="s">
@@ -3547,14 +3547,14 @@
       <c r="AT2" s="72"/>
     </row>
     <row r="3" spans="1:46" ht="33" customHeight="1">
-      <c r="A3" s="76"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="73" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
       <c r="G3" s="72" t="s">
         <v>16</v>
       </c>
@@ -3599,57 +3599,57 @@
       <c r="AT3" s="72"/>
     </row>
     <row r="4" spans="1:46" ht="21">
-      <c r="A4" s="76"/>
-      <c r="B4" s="78"/>
-      <c r="C4" s="73" t="s">
+      <c r="A4" s="69"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="78" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="73" t="s">
+      <c r="E4" s="78" t="s">
         <v>19</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="73" t="s">
+      <c r="G4" s="78" t="s">
         <v>17</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="69" t="s">
+      <c r="K4" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="71"/>
-      <c r="Q4" s="69" t="s">
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="77"/>
+      <c r="Q4" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="70"/>
-      <c r="S4" s="70"/>
-      <c r="T4" s="70"/>
-      <c r="U4" s="70"/>
-      <c r="V4" s="70"/>
-      <c r="W4" s="70"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="70"/>
-      <c r="Z4" s="70"/>
-      <c r="AA4" s="70"/>
-      <c r="AB4" s="70"/>
-      <c r="AC4" s="70"/>
-      <c r="AD4" s="70"/>
-      <c r="AE4" s="71"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="76"/>
+      <c r="Z4" s="76"/>
+      <c r="AA4" s="76"/>
+      <c r="AB4" s="76"/>
+      <c r="AC4" s="76"/>
+      <c r="AD4" s="76"/>
+      <c r="AE4" s="77"/>
       <c r="AF4" s="72" t="s">
         <v>24</v>
       </c>
@@ -3669,22 +3669,22 @@
       <c r="AT4" s="72"/>
     </row>
     <row r="5" spans="1:46">
-      <c r="A5" s="77"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="73"/>
+      <c r="A5" s="70"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="78"/>
       <c r="D5" s="13">
         <v>2025</v>
       </c>
-      <c r="E5" s="73"/>
+      <c r="E5" s="78"/>
       <c r="F5" s="13">
         <v>2025</v>
       </c>
-      <c r="G5" s="73"/>
+      <c r="G5" s="78"/>
       <c r="H5" s="13">
         <v>2025</v>
       </c>
-      <c r="I5" s="73"/>
-      <c r="J5" s="68"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="74"/>
       <c r="K5" s="13">
         <v>1990</v>
       </c>
@@ -32551,7 +32551,7 @@
         <v>480</v>
       </c>
       <c r="B230" s="16" t="s">
-        <v>481</v>
+        <v>533</v>
       </c>
       <c r="C230" s="17"/>
       <c r="D230" s="19"/>
@@ -32676,10 +32676,10 @@
     </row>
     <row r="231" spans="1:46" outlineLevel="1">
       <c r="A231" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="B231" s="16" t="s">
         <v>482</v>
-      </c>
-      <c r="B231" s="16" t="s">
-        <v>483</v>
       </c>
       <c r="C231" s="17"/>
       <c r="D231" s="19"/>
@@ -32804,10 +32804,10 @@
     </row>
     <row r="232" spans="1:46" outlineLevel="1">
       <c r="A232" s="15" t="s">
+        <v>483</v>
+      </c>
+      <c r="B232" s="16" t="s">
         <v>484</v>
-      </c>
-      <c r="B232" s="16" t="s">
-        <v>485</v>
       </c>
       <c r="C232" s="17"/>
       <c r="D232" s="19"/>
@@ -32932,10 +32932,10 @@
     </row>
     <row r="233" spans="1:46" outlineLevel="1">
       <c r="A233" s="15" t="s">
+        <v>485</v>
+      </c>
+      <c r="B233" s="16" t="s">
         <v>486</v>
-      </c>
-      <c r="B233" s="16" t="s">
-        <v>487</v>
       </c>
       <c r="C233" s="17"/>
       <c r="D233" s="19"/>
@@ -33060,10 +33060,10 @@
     </row>
     <row r="234" spans="1:46" outlineLevel="1">
       <c r="A234" s="15" t="s">
+        <v>487</v>
+      </c>
+      <c r="B234" s="16" t="s">
         <v>488</v>
-      </c>
-      <c r="B234" s="16" t="s">
-        <v>489</v>
       </c>
       <c r="C234" s="17"/>
       <c r="D234" s="19"/>
@@ -33188,10 +33188,10 @@
     </row>
     <row r="235" spans="1:46" outlineLevel="1">
       <c r="A235" s="15" t="s">
+        <v>489</v>
+      </c>
+      <c r="B235" s="16" t="s">
         <v>490</v>
-      </c>
-      <c r="B235" s="16" t="s">
-        <v>491</v>
       </c>
       <c r="C235" s="17"/>
       <c r="D235" s="19"/>
@@ -33316,10 +33316,10 @@
     </row>
     <row r="236" spans="1:46" outlineLevel="1">
       <c r="A236" s="15" t="s">
+        <v>491</v>
+      </c>
+      <c r="B236" s="16" t="s">
         <v>492</v>
-      </c>
-      <c r="B236" s="16" t="s">
-        <v>493</v>
       </c>
       <c r="C236" s="17"/>
       <c r="D236" s="19"/>
@@ -33444,10 +33444,10 @@
     </row>
     <row r="237" spans="1:46" outlineLevel="1">
       <c r="A237" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="B237" s="16" t="s">
         <v>494</v>
-      </c>
-      <c r="B237" s="16" t="s">
-        <v>495</v>
       </c>
       <c r="C237" s="17"/>
       <c r="D237" s="19"/>
@@ -33708,10 +33708,10 @@
     </row>
     <row r="239" spans="1:46" outlineLevel="1">
       <c r="A239" s="15" t="s">
+        <v>495</v>
+      </c>
+      <c r="B239" s="16" t="s">
         <v>496</v>
-      </c>
-      <c r="B239" s="16" t="s">
-        <v>497</v>
       </c>
       <c r="C239" s="17"/>
       <c r="D239" s="19"/>
@@ -33836,10 +33836,10 @@
     </row>
     <row r="240" spans="1:46" outlineLevel="1">
       <c r="A240" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="B240" s="16" t="s">
         <v>499</v>
-      </c>
-      <c r="B240" s="16" t="s">
-        <v>500</v>
       </c>
       <c r="C240" s="17"/>
       <c r="D240" s="19"/>
@@ -33964,10 +33964,10 @@
     </row>
     <row r="241" spans="1:46" outlineLevel="1">
       <c r="A241" s="15" t="s">
+        <v>500</v>
+      </c>
+      <c r="B241" s="16" t="s">
         <v>501</v>
-      </c>
-      <c r="B241" s="16" t="s">
-        <v>502</v>
       </c>
       <c r="C241" s="17"/>
       <c r="D241" s="19"/>
@@ -34092,10 +34092,10 @@
     </row>
     <row r="242" spans="1:46" outlineLevel="1">
       <c r="A242" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="B242" s="16" t="s">
         <v>503</v>
-      </c>
-      <c r="B242" s="16" t="s">
-        <v>504</v>
       </c>
       <c r="C242" s="17"/>
       <c r="D242" s="19"/>
@@ -34220,10 +34220,10 @@
     </row>
     <row r="243" spans="1:46" outlineLevel="1">
       <c r="A243" s="15" t="s">
+        <v>504</v>
+      </c>
+      <c r="B243" s="16" t="s">
         <v>505</v>
-      </c>
-      <c r="B243" s="16" t="s">
-        <v>506</v>
       </c>
       <c r="C243" s="17"/>
       <c r="D243" s="19"/>
@@ -34348,10 +34348,10 @@
     </row>
     <row r="244" spans="1:46" outlineLevel="1">
       <c r="A244" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="B244" s="16" t="s">
         <v>507</v>
-      </c>
-      <c r="B244" s="16" t="s">
-        <v>508</v>
       </c>
       <c r="C244" s="17"/>
       <c r="D244" s="19"/>
@@ -34476,10 +34476,10 @@
     </row>
     <row r="245" spans="1:46" outlineLevel="1">
       <c r="A245" s="15" t="s">
+        <v>508</v>
+      </c>
+      <c r="B245" s="16" t="s">
         <v>509</v>
-      </c>
-      <c r="B245" s="16" t="s">
-        <v>510</v>
       </c>
       <c r="C245" s="17"/>
       <c r="D245" s="19"/>
@@ -34604,10 +34604,10 @@
     </row>
     <row r="246" spans="1:46" outlineLevel="1">
       <c r="A246" s="15" t="s">
+        <v>510</v>
+      </c>
+      <c r="B246" s="16" t="s">
         <v>511</v>
-      </c>
-      <c r="B246" s="16" t="s">
-        <v>512</v>
       </c>
       <c r="C246" s="17"/>
       <c r="D246" s="19"/>
@@ -34732,10 +34732,10 @@
     </row>
     <row r="247" spans="1:46" outlineLevel="1">
       <c r="A247" s="15" t="s">
+        <v>512</v>
+      </c>
+      <c r="B247" s="16" t="s">
         <v>513</v>
-      </c>
-      <c r="B247" s="16" t="s">
-        <v>514</v>
       </c>
       <c r="C247" s="17"/>
       <c r="D247" s="19"/>
@@ -34860,10 +34860,10 @@
     </row>
     <row r="248" spans="1:46" outlineLevel="1">
       <c r="A248" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="B248" s="16" t="s">
         <v>515</v>
-      </c>
-      <c r="B248" s="16" t="s">
-        <v>516</v>
       </c>
       <c r="C248" s="17"/>
       <c r="D248" s="19"/>
@@ -34988,10 +34988,10 @@
     </row>
     <row r="249" spans="1:46" outlineLevel="1">
       <c r="A249" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B249" s="16" t="s">
         <v>517</v>
-      </c>
-      <c r="B249" s="16" t="s">
-        <v>518</v>
       </c>
       <c r="C249" s="17"/>
       <c r="D249" s="19"/>
@@ -35116,10 +35116,10 @@
     </row>
     <row r="250" spans="1:46" outlineLevel="1">
       <c r="A250" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="B250" s="16" t="s">
         <v>519</v>
-      </c>
-      <c r="B250" s="16" t="s">
-        <v>520</v>
       </c>
       <c r="C250" s="17"/>
       <c r="D250" s="19"/>
@@ -35244,10 +35244,10 @@
     </row>
     <row r="251" spans="1:46" outlineLevel="1">
       <c r="A251" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="B251" s="16" t="s">
         <v>521</v>
-      </c>
-      <c r="B251" s="16" t="s">
-        <v>522</v>
       </c>
       <c r="C251" s="17"/>
       <c r="D251" s="19"/>
@@ -35372,10 +35372,10 @@
     </row>
     <row r="252" spans="1:46" outlineLevel="1">
       <c r="A252" s="15" t="s">
+        <v>522</v>
+      </c>
+      <c r="B252" s="16" t="s">
         <v>523</v>
-      </c>
-      <c r="B252" s="16" t="s">
-        <v>524</v>
       </c>
       <c r="C252" s="17"/>
       <c r="D252" s="19"/>
@@ -35501,7 +35501,7 @@
     <row r="253" spans="1:46" s="9" customFormat="1" ht="15" thickBot="1">
       <c r="A253" s="30"/>
       <c r="B253" s="31" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C253" s="32">
         <v>11</v>
@@ -35637,7 +35637,7 @@
     <row r="254" spans="1:46" s="9" customFormat="1" ht="26.25" customHeight="1">
       <c r="A254" s="37"/>
       <c r="B254" s="38" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C254" s="39">
         <v>141</v>
@@ -35773,7 +35773,7 @@
     <row r="255" spans="1:46" s="9" customFormat="1">
       <c r="A255" s="49"/>
       <c r="B255" s="50" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C255" s="51">
         <v>43</v>
@@ -35909,7 +35909,7 @@
     <row r="256" spans="1:46" s="9" customFormat="1">
       <c r="A256" s="49"/>
       <c r="B256" s="50" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C256" s="51">
         <v>29</v>
@@ -36181,7 +36181,7 @@
     <row r="258" spans="1:46" s="9" customFormat="1">
       <c r="A258" s="49"/>
       <c r="B258" s="50" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C258" s="51">
         <v>21</v>
@@ -36453,7 +36453,7 @@
     <row r="260" spans="1:46" s="9" customFormat="1">
       <c r="A260" s="49"/>
       <c r="B260" s="50" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C260" s="51">
         <v>11</v>

</xml_diff>

<commit_message>
5417 - Static file upload: --reupload and update bulk download files (#5428)
</commit_message>
<xml_diff>
--- a/src/tools/uploadStaticFiles/staticFiles/fra/2025/dataDownload/6 Permanent forest estate en.xlsx
+++ b/src/tools/uploadStaticFiles/staticFiles/fra/2025/dataDownload/6 Permanent forest estate en.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29231"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfao-my.sharepoint.com/personal/pengcheng_lai_fao_org/Documents/Desktop/worksheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://unfao-my.sharepoint.com/personal/pengcheng_lai_fao_org/Documents/Desktop/Update/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="8_{9EB7299C-8445-45FA-928C-21125EB2985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2B78550D-900F-47F3-94D3-702C715DA43D}"/>
+  <xr:revisionPtr revIDLastSave="17" documentId="8_{9EB7299C-8445-45FA-928C-21125EB2985C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{06A64972-452A-46DE-ABA1-0DD5BCE4B625}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1670,9 +1670,6 @@
     <t>PCN</t>
   </si>
   <si>
-    <t>Pitcairn Islands</t>
-  </si>
-  <si>
     <t>WSM</t>
   </si>
   <si>
@@ -1879,6 +1876,9 @@
   </si>
   <si>
     <t>These analysis tables include data reported by countries and it is important to note that some of the regional totals may differ from the results presented in the FRA 2025 main report. The reason for this discrepancy is that in some cases, gap-filling was performed for missing values in order to obtain complete time series for the main report. Therefore, it is not always possible to reproduce the global, regional and subregional aggregates presented in the FRA 2025 main report by using the analysis tables.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Pitcairn </t>
   </si>
 </sst>
 </file>
@@ -2396,6 +2396,24 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2412,25 +2430,7 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3088,7 +3088,7 @@
     </row>
     <row r="2" spans="1:17" ht="15.75" customHeight="1">
       <c r="A2" s="64" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="B2" s="64"/>
       <c r="C2" s="64"/>
@@ -3149,7 +3149,7 @@
     </row>
     <row r="5" spans="1:17" ht="32.25" customHeight="1">
       <c r="A5" s="64" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="B5" s="64"/>
       <c r="C5" s="64"/>
@@ -3191,7 +3191,7 @@
     </row>
     <row r="7" spans="1:17" ht="48" customHeight="1">
       <c r="A7" s="61" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="B7" s="61"/>
       <c r="C7" s="61"/>
@@ -3254,7 +3254,7 @@
     </row>
     <row r="10" spans="1:17">
       <c r="A10" s="63" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="B10" s="63"/>
       <c r="C10" s="63"/>
@@ -3363,17 +3363,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A7:Q7"/>
-    <mergeCell ref="A8:Q8"/>
-    <mergeCell ref="A9:Q9"/>
-    <mergeCell ref="A10:Q10"/>
-    <mergeCell ref="A83:Q83"/>
     <mergeCell ref="A89:Q89"/>
     <mergeCell ref="A1:Q1"/>
     <mergeCell ref="A2:Q3"/>
     <mergeCell ref="A4:Q4"/>
     <mergeCell ref="A5:Q5"/>
     <mergeCell ref="A6:Q6"/>
+    <mergeCell ref="A7:Q7"/>
+    <mergeCell ref="A8:Q8"/>
+    <mergeCell ref="A9:Q9"/>
+    <mergeCell ref="A10:Q10"/>
+    <mergeCell ref="A83:Q83"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -3439,62 +3439,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:46" s="7" customFormat="1" ht="24" customHeight="1">
-      <c r="A1" s="74" t="s">
+      <c r="A1" s="67" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="74"/>
-      <c r="C1" s="74" t="s">
-        <v>529</v>
-      </c>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="74"/>
-      <c r="L1" s="74"/>
-      <c r="M1" s="74"/>
-      <c r="N1" s="74"/>
-      <c r="O1" s="74"/>
-      <c r="P1" s="74"/>
-      <c r="Q1" s="74"/>
-      <c r="R1" s="74"/>
-      <c r="S1" s="74"/>
-      <c r="T1" s="74"/>
-      <c r="U1" s="74"/>
-      <c r="V1" s="74"/>
-      <c r="W1" s="74"/>
-      <c r="X1" s="74"/>
-      <c r="Y1" s="74"/>
-      <c r="Z1" s="74"/>
-      <c r="AA1" s="74"/>
-      <c r="AB1" s="74"/>
-      <c r="AC1" s="74"/>
-      <c r="AD1" s="74"/>
-      <c r="AE1" s="74"/>
-      <c r="AF1" s="74"/>
-      <c r="AG1" s="74"/>
-      <c r="AH1" s="74"/>
-      <c r="AI1" s="74"/>
-      <c r="AJ1" s="74"/>
-      <c r="AK1" s="74"/>
-      <c r="AL1" s="74"/>
-      <c r="AM1" s="74"/>
-      <c r="AN1" s="74"/>
-      <c r="AO1" s="74"/>
-      <c r="AP1" s="74"/>
-      <c r="AQ1" s="74"/>
-      <c r="AR1" s="74"/>
-      <c r="AS1" s="74"/>
-      <c r="AT1" s="74"/>
+      <c r="B1" s="67"/>
+      <c r="C1" s="67" t="s">
+        <v>528</v>
+      </c>
+      <c r="D1" s="67"/>
+      <c r="E1" s="67"/>
+      <c r="F1" s="67"/>
+      <c r="G1" s="67"/>
+      <c r="H1" s="67"/>
+      <c r="I1" s="67"/>
+      <c r="J1" s="67"/>
+      <c r="K1" s="67"/>
+      <c r="L1" s="67"/>
+      <c r="M1" s="67"/>
+      <c r="N1" s="67"/>
+      <c r="O1" s="67"/>
+      <c r="P1" s="67"/>
+      <c r="Q1" s="67"/>
+      <c r="R1" s="67"/>
+      <c r="S1" s="67"/>
+      <c r="T1" s="67"/>
+      <c r="U1" s="67"/>
+      <c r="V1" s="67"/>
+      <c r="W1" s="67"/>
+      <c r="X1" s="67"/>
+      <c r="Y1" s="67"/>
+      <c r="Z1" s="67"/>
+      <c r="AA1" s="67"/>
+      <c r="AB1" s="67"/>
+      <c r="AC1" s="67"/>
+      <c r="AD1" s="67"/>
+      <c r="AE1" s="67"/>
+      <c r="AF1" s="67"/>
+      <c r="AG1" s="67"/>
+      <c r="AH1" s="67"/>
+      <c r="AI1" s="67"/>
+      <c r="AJ1" s="67"/>
+      <c r="AK1" s="67"/>
+      <c r="AL1" s="67"/>
+      <c r="AM1" s="67"/>
+      <c r="AN1" s="67"/>
+      <c r="AO1" s="67"/>
+      <c r="AP1" s="67"/>
+      <c r="AQ1" s="67"/>
+      <c r="AR1" s="67"/>
+      <c r="AS1" s="67"/>
+      <c r="AT1" s="67"/>
     </row>
     <row r="2" spans="1:46">
-      <c r="A2" s="75" t="s">
+      <c r="A2" s="68" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="78" t="s">
+      <c r="B2" s="71" t="s">
         <v>12</v>
       </c>
       <c r="C2" s="72" t="s">
@@ -3547,14 +3547,14 @@
       <c r="AT2" s="72"/>
     </row>
     <row r="3" spans="1:46" ht="33" customHeight="1">
-      <c r="A3" s="76"/>
-      <c r="B3" s="78"/>
-      <c r="C3" s="73" t="s">
+      <c r="A3" s="69"/>
+      <c r="B3" s="71"/>
+      <c r="C3" s="78" t="s">
         <v>15</v>
       </c>
-      <c r="D3" s="73"/>
-      <c r="E3" s="73"/>
-      <c r="F3" s="73"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="78"/>
+      <c r="F3" s="78"/>
       <c r="G3" s="72" t="s">
         <v>16</v>
       </c>
@@ -3599,57 +3599,57 @@
       <c r="AT3" s="72"/>
     </row>
     <row r="4" spans="1:46" ht="21">
-      <c r="A4" s="76"/>
-      <c r="B4" s="78"/>
-      <c r="C4" s="73" t="s">
+      <c r="A4" s="69"/>
+      <c r="B4" s="71"/>
+      <c r="C4" s="78" t="s">
         <v>17</v>
       </c>
       <c r="D4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E4" s="73" t="s">
+      <c r="E4" s="78" t="s">
         <v>19</v>
       </c>
       <c r="F4" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="G4" s="73" t="s">
+      <c r="G4" s="78" t="s">
         <v>17</v>
       </c>
       <c r="H4" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="I4" s="73" t="s">
+      <c r="I4" s="78" t="s">
         <v>19</v>
       </c>
-      <c r="J4" s="67" t="s">
+      <c r="J4" s="73" t="s">
         <v>21</v>
       </c>
-      <c r="K4" s="69" t="s">
+      <c r="K4" s="75" t="s">
         <v>22</v>
       </c>
-      <c r="L4" s="70"/>
-      <c r="M4" s="70"/>
-      <c r="N4" s="70"/>
-      <c r="O4" s="70"/>
-      <c r="P4" s="71"/>
-      <c r="Q4" s="69" t="s">
+      <c r="L4" s="76"/>
+      <c r="M4" s="76"/>
+      <c r="N4" s="76"/>
+      <c r="O4" s="76"/>
+      <c r="P4" s="77"/>
+      <c r="Q4" s="75" t="s">
         <v>23</v>
       </c>
-      <c r="R4" s="70"/>
-      <c r="S4" s="70"/>
-      <c r="T4" s="70"/>
-      <c r="U4" s="70"/>
-      <c r="V4" s="70"/>
-      <c r="W4" s="70"/>
-      <c r="X4" s="70"/>
-      <c r="Y4" s="70"/>
-      <c r="Z4" s="70"/>
-      <c r="AA4" s="70"/>
-      <c r="AB4" s="70"/>
-      <c r="AC4" s="70"/>
-      <c r="AD4" s="70"/>
-      <c r="AE4" s="71"/>
+      <c r="R4" s="76"/>
+      <c r="S4" s="76"/>
+      <c r="T4" s="76"/>
+      <c r="U4" s="76"/>
+      <c r="V4" s="76"/>
+      <c r="W4" s="76"/>
+      <c r="X4" s="76"/>
+      <c r="Y4" s="76"/>
+      <c r="Z4" s="76"/>
+      <c r="AA4" s="76"/>
+      <c r="AB4" s="76"/>
+      <c r="AC4" s="76"/>
+      <c r="AD4" s="76"/>
+      <c r="AE4" s="77"/>
       <c r="AF4" s="72" t="s">
         <v>24</v>
       </c>
@@ -3669,22 +3669,22 @@
       <c r="AT4" s="72"/>
     </row>
     <row r="5" spans="1:46">
-      <c r="A5" s="77"/>
-      <c r="B5" s="78"/>
-      <c r="C5" s="73"/>
+      <c r="A5" s="70"/>
+      <c r="B5" s="71"/>
+      <c r="C5" s="78"/>
       <c r="D5" s="13">
         <v>2025</v>
       </c>
-      <c r="E5" s="73"/>
+      <c r="E5" s="78"/>
       <c r="F5" s="13">
         <v>2025</v>
       </c>
-      <c r="G5" s="73"/>
+      <c r="G5" s="78"/>
       <c r="H5" s="13">
         <v>2025</v>
       </c>
-      <c r="I5" s="73"/>
-      <c r="J5" s="68"/>
+      <c r="I5" s="78"/>
+      <c r="J5" s="74"/>
       <c r="K5" s="13">
         <v>1990</v>
       </c>
@@ -32551,7 +32551,7 @@
         <v>480</v>
       </c>
       <c r="B230" s="16" t="s">
-        <v>481</v>
+        <v>533</v>
       </c>
       <c r="C230" s="17"/>
       <c r="D230" s="19"/>
@@ -32676,10 +32676,10 @@
     </row>
     <row r="231" spans="1:46" outlineLevel="1">
       <c r="A231" s="15" t="s">
+        <v>481</v>
+      </c>
+      <c r="B231" s="16" t="s">
         <v>482</v>
-      </c>
-      <c r="B231" s="16" t="s">
-        <v>483</v>
       </c>
       <c r="C231" s="17"/>
       <c r="D231" s="19"/>
@@ -32804,10 +32804,10 @@
     </row>
     <row r="232" spans="1:46" outlineLevel="1">
       <c r="A232" s="15" t="s">
+        <v>483</v>
+      </c>
+      <c r="B232" s="16" t="s">
         <v>484</v>
-      </c>
-      <c r="B232" s="16" t="s">
-        <v>485</v>
       </c>
       <c r="C232" s="17"/>
       <c r="D232" s="19"/>
@@ -32932,10 +32932,10 @@
     </row>
     <row r="233" spans="1:46" outlineLevel="1">
       <c r="A233" s="15" t="s">
+        <v>485</v>
+      </c>
+      <c r="B233" s="16" t="s">
         <v>486</v>
-      </c>
-      <c r="B233" s="16" t="s">
-        <v>487</v>
       </c>
       <c r="C233" s="17"/>
       <c r="D233" s="19"/>
@@ -33060,10 +33060,10 @@
     </row>
     <row r="234" spans="1:46" outlineLevel="1">
       <c r="A234" s="15" t="s">
+        <v>487</v>
+      </c>
+      <c r="B234" s="16" t="s">
         <v>488</v>
-      </c>
-      <c r="B234" s="16" t="s">
-        <v>489</v>
       </c>
       <c r="C234" s="17"/>
       <c r="D234" s="19"/>
@@ -33188,10 +33188,10 @@
     </row>
     <row r="235" spans="1:46" outlineLevel="1">
       <c r="A235" s="15" t="s">
+        <v>489</v>
+      </c>
+      <c r="B235" s="16" t="s">
         <v>490</v>
-      </c>
-      <c r="B235" s="16" t="s">
-        <v>491</v>
       </c>
       <c r="C235" s="17"/>
       <c r="D235" s="19"/>
@@ -33316,10 +33316,10 @@
     </row>
     <row r="236" spans="1:46" outlineLevel="1">
       <c r="A236" s="15" t="s">
+        <v>491</v>
+      </c>
+      <c r="B236" s="16" t="s">
         <v>492</v>
-      </c>
-      <c r="B236" s="16" t="s">
-        <v>493</v>
       </c>
       <c r="C236" s="17"/>
       <c r="D236" s="19"/>
@@ -33444,10 +33444,10 @@
     </row>
     <row r="237" spans="1:46" outlineLevel="1">
       <c r="A237" s="15" t="s">
+        <v>493</v>
+      </c>
+      <c r="B237" s="16" t="s">
         <v>494</v>
-      </c>
-      <c r="B237" s="16" t="s">
-        <v>495</v>
       </c>
       <c r="C237" s="17"/>
       <c r="D237" s="19"/>
@@ -33708,10 +33708,10 @@
     </row>
     <row r="239" spans="1:46" outlineLevel="1">
       <c r="A239" s="15" t="s">
+        <v>495</v>
+      </c>
+      <c r="B239" s="16" t="s">
         <v>496</v>
-      </c>
-      <c r="B239" s="16" t="s">
-        <v>497</v>
       </c>
       <c r="C239" s="17"/>
       <c r="D239" s="19"/>
@@ -33836,10 +33836,10 @@
     </row>
     <row r="240" spans="1:46" outlineLevel="1">
       <c r="A240" s="15" t="s">
+        <v>498</v>
+      </c>
+      <c r="B240" s="16" t="s">
         <v>499</v>
-      </c>
-      <c r="B240" s="16" t="s">
-        <v>500</v>
       </c>
       <c r="C240" s="17"/>
       <c r="D240" s="19"/>
@@ -33964,10 +33964,10 @@
     </row>
     <row r="241" spans="1:46" outlineLevel="1">
       <c r="A241" s="15" t="s">
+        <v>500</v>
+      </c>
+      <c r="B241" s="16" t="s">
         <v>501</v>
-      </c>
-      <c r="B241" s="16" t="s">
-        <v>502</v>
       </c>
       <c r="C241" s="17"/>
       <c r="D241" s="19"/>
@@ -34092,10 +34092,10 @@
     </row>
     <row r="242" spans="1:46" outlineLevel="1">
       <c r="A242" s="15" t="s">
+        <v>502</v>
+      </c>
+      <c r="B242" s="16" t="s">
         <v>503</v>
-      </c>
-      <c r="B242" s="16" t="s">
-        <v>504</v>
       </c>
       <c r="C242" s="17"/>
       <c r="D242" s="19"/>
@@ -34220,10 +34220,10 @@
     </row>
     <row r="243" spans="1:46" outlineLevel="1">
       <c r="A243" s="15" t="s">
+        <v>504</v>
+      </c>
+      <c r="B243" s="16" t="s">
         <v>505</v>
-      </c>
-      <c r="B243" s="16" t="s">
-        <v>506</v>
       </c>
       <c r="C243" s="17"/>
       <c r="D243" s="19"/>
@@ -34348,10 +34348,10 @@
     </row>
     <row r="244" spans="1:46" outlineLevel="1">
       <c r="A244" s="15" t="s">
+        <v>506</v>
+      </c>
+      <c r="B244" s="16" t="s">
         <v>507</v>
-      </c>
-      <c r="B244" s="16" t="s">
-        <v>508</v>
       </c>
       <c r="C244" s="17"/>
       <c r="D244" s="19"/>
@@ -34476,10 +34476,10 @@
     </row>
     <row r="245" spans="1:46" outlineLevel="1">
       <c r="A245" s="15" t="s">
+        <v>508</v>
+      </c>
+      <c r="B245" s="16" t="s">
         <v>509</v>
-      </c>
-      <c r="B245" s="16" t="s">
-        <v>510</v>
       </c>
       <c r="C245" s="17"/>
       <c r="D245" s="19"/>
@@ -34604,10 +34604,10 @@
     </row>
     <row r="246" spans="1:46" outlineLevel="1">
       <c r="A246" s="15" t="s">
+        <v>510</v>
+      </c>
+      <c r="B246" s="16" t="s">
         <v>511</v>
-      </c>
-      <c r="B246" s="16" t="s">
-        <v>512</v>
       </c>
       <c r="C246" s="17"/>
       <c r="D246" s="19"/>
@@ -34732,10 +34732,10 @@
     </row>
     <row r="247" spans="1:46" outlineLevel="1">
       <c r="A247" s="15" t="s">
+        <v>512</v>
+      </c>
+      <c r="B247" s="16" t="s">
         <v>513</v>
-      </c>
-      <c r="B247" s="16" t="s">
-        <v>514</v>
       </c>
       <c r="C247" s="17"/>
       <c r="D247" s="19"/>
@@ -34860,10 +34860,10 @@
     </row>
     <row r="248" spans="1:46" outlineLevel="1">
       <c r="A248" s="15" t="s">
+        <v>514</v>
+      </c>
+      <c r="B248" s="16" t="s">
         <v>515</v>
-      </c>
-      <c r="B248" s="16" t="s">
-        <v>516</v>
       </c>
       <c r="C248" s="17"/>
       <c r="D248" s="19"/>
@@ -34988,10 +34988,10 @@
     </row>
     <row r="249" spans="1:46" outlineLevel="1">
       <c r="A249" s="15" t="s">
+        <v>516</v>
+      </c>
+      <c r="B249" s="16" t="s">
         <v>517</v>
-      </c>
-      <c r="B249" s="16" t="s">
-        <v>518</v>
       </c>
       <c r="C249" s="17"/>
       <c r="D249" s="19"/>
@@ -35116,10 +35116,10 @@
     </row>
     <row r="250" spans="1:46" outlineLevel="1">
       <c r="A250" s="15" t="s">
+        <v>518</v>
+      </c>
+      <c r="B250" s="16" t="s">
         <v>519</v>
-      </c>
-      <c r="B250" s="16" t="s">
-        <v>520</v>
       </c>
       <c r="C250" s="17"/>
       <c r="D250" s="19"/>
@@ -35244,10 +35244,10 @@
     </row>
     <row r="251" spans="1:46" outlineLevel="1">
       <c r="A251" s="15" t="s">
+        <v>520</v>
+      </c>
+      <c r="B251" s="16" t="s">
         <v>521</v>
-      </c>
-      <c r="B251" s="16" t="s">
-        <v>522</v>
       </c>
       <c r="C251" s="17"/>
       <c r="D251" s="19"/>
@@ -35372,10 +35372,10 @@
     </row>
     <row r="252" spans="1:46" outlineLevel="1">
       <c r="A252" s="15" t="s">
+        <v>522</v>
+      </c>
+      <c r="B252" s="16" t="s">
         <v>523</v>
-      </c>
-      <c r="B252" s="16" t="s">
-        <v>524</v>
       </c>
       <c r="C252" s="17"/>
       <c r="D252" s="19"/>
@@ -35501,7 +35501,7 @@
     <row r="253" spans="1:46" s="9" customFormat="1" ht="15" thickBot="1">
       <c r="A253" s="30"/>
       <c r="B253" s="31" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C253" s="32">
         <v>11</v>
@@ -35637,7 +35637,7 @@
     <row r="254" spans="1:46" s="9" customFormat="1" ht="26.25" customHeight="1">
       <c r="A254" s="37"/>
       <c r="B254" s="38" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="C254" s="39">
         <v>141</v>
@@ -35773,7 +35773,7 @@
     <row r="255" spans="1:46" s="9" customFormat="1">
       <c r="A255" s="49"/>
       <c r="B255" s="50" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="C255" s="51">
         <v>43</v>
@@ -35909,7 +35909,7 @@
     <row r="256" spans="1:46" s="9" customFormat="1">
       <c r="A256" s="49"/>
       <c r="B256" s="50" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="C256" s="51">
         <v>29</v>
@@ -36181,7 +36181,7 @@
     <row r="258" spans="1:46" s="9" customFormat="1">
       <c r="A258" s="49"/>
       <c r="B258" s="50" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="C258" s="51">
         <v>21</v>
@@ -36453,7 +36453,7 @@
     <row r="260" spans="1:46" s="9" customFormat="1">
       <c r="A260" s="49"/>
       <c r="B260" s="50" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="C260" s="51">
         <v>11</v>

</xml_diff>